<commit_message>
updated boq generator file
</commit_message>
<xml_diff>
--- a/boq_plain.xlsx
+++ b/boq_plain.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -483,12 +483,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Floor Finish</t>
+          <t>Floor Finishes</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Floor tiling to AD-02</t>
+          <t>Floor tiling</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -497,13 +497,13 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>8.699999999999999</v>
+        <v>89.56</v>
       </c>
       <c r="G2" t="n">
         <v>15000</v>
       </c>
       <c r="H2" t="n">
-        <v>130500</v>
+        <v>1343400</v>
       </c>
     </row>
     <row r="3">
@@ -519,12 +519,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Wall Finish</t>
+          <t>Wall Finishes</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Plastering to walls in AD-02</t>
+          <t>Plastering to walls</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -533,13 +533,13 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>48.2</v>
+        <v>163.66</v>
       </c>
       <c r="G3" t="n">
         <v>12000</v>
       </c>
       <c r="H3" t="n">
-        <v>578400</v>
+        <v>1963920</v>
       </c>
     </row>
     <row r="4">
@@ -555,27 +555,27 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>Skirtings</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>Skirting</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Skirting to AD-02</t>
-        </is>
-      </c>
       <c r="E4" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>13.39</v>
+        <v>49.36</v>
       </c>
       <c r="G4" t="n">
         <v>2500</v>
       </c>
       <c r="H4" t="n">
-        <v>33475</v>
+        <v>123400</v>
       </c>
     </row>
     <row r="5">
@@ -591,12 +591,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Ceiling Finish</t>
+          <t>Ceiling Finishes</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Ceiling finish to AD-02</t>
+          <t>Ceiling finish</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -605,157 +605,13 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>8.699999999999999</v>
+        <v>89.56</v>
       </c>
       <c r="G5" t="n">
         <v>10000</v>
       </c>
       <c r="H5" t="n">
-        <v>87000</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Finishes</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Floor Finish</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Floor tiling to A</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="F6" t="n">
-        <v>80.86</v>
-      </c>
-      <c r="G6" t="n">
-        <v>15000</v>
-      </c>
-      <c r="H6" t="n">
-        <v>1212900</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Finishes</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Wall Finish</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Plastering to walls in A</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="F7" t="n">
-        <v>115.46</v>
-      </c>
-      <c r="G7" t="n">
-        <v>12000</v>
-      </c>
-      <c r="H7" t="n">
-        <v>1385520</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Finishes</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Skirting</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Skirting to A</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="F8" t="n">
-        <v>35.97</v>
-      </c>
-      <c r="G8" t="n">
-        <v>2500</v>
-      </c>
-      <c r="H8" t="n">
-        <v>89925</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>H</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Finishes</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Ceiling Finish</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Ceiling finish to A</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="F9" t="n">
-        <v>80.86</v>
-      </c>
-      <c r="G9" t="n">
-        <v>10000</v>
-      </c>
-      <c r="H9" t="n">
-        <v>808600</v>
+        <v>895600</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update ai pricing file
</commit_message>
<xml_diff>
--- a/boq_plain.xlsx
+++ b/boq_plain.xlsx
@@ -500,7 +500,7 @@
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>30000</v>
+        <v>35000</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
@@ -536,7 +536,7 @@
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>35000</v>
+        <v>38000</v>
       </c>
       <c r="H3" t="n">
         <v>0</v>
@@ -572,10 +572,10 @@
         <v>444</v>
       </c>
       <c r="G4" t="n">
-        <v>40000</v>
+        <v>42000</v>
       </c>
       <c r="H4" t="n">
-        <v>17760000</v>
+        <v>18648000</v>
       </c>
     </row>
     <row r="5">
@@ -608,10 +608,10 @@
         <v>370</v>
       </c>
       <c r="G5" t="n">
-        <v>40000</v>
+        <v>42000</v>
       </c>
       <c r="H5" t="n">
-        <v>14800000</v>
+        <v>15540000</v>
       </c>
     </row>
     <row r="6">
@@ -644,10 +644,10 @@
         <v>370</v>
       </c>
       <c r="G6" t="n">
-        <v>40000</v>
+        <v>42000</v>
       </c>
       <c r="H6" t="n">
-        <v>14800000</v>
+        <v>15540000</v>
       </c>
     </row>
     <row r="7">
@@ -680,10 +680,10 @@
         <v>74</v>
       </c>
       <c r="G7" t="n">
-        <v>40000</v>
+        <v>42000</v>
       </c>
       <c r="H7" t="n">
-        <v>2960000</v>
+        <v>3108000</v>
       </c>
     </row>
     <row r="8">
@@ -716,10 +716,10 @@
         <v>370</v>
       </c>
       <c r="G8" t="n">
-        <v>45000</v>
+        <v>50000</v>
       </c>
       <c r="H8" t="n">
-        <v>16650000</v>
+        <v>18500000</v>
       </c>
     </row>
     <row r="9">
@@ -752,10 +752,10 @@
         <v>74</v>
       </c>
       <c r="G9" t="n">
-        <v>40000</v>
+        <v>42000</v>
       </c>
       <c r="H9" t="n">
-        <v>2960000</v>
+        <v>3108000</v>
       </c>
     </row>
     <row r="10">
@@ -788,10 +788,10 @@
         <v>518</v>
       </c>
       <c r="G10" t="n">
-        <v>45000</v>
+        <v>50000</v>
       </c>
       <c r="H10" t="n">
-        <v>23310000</v>
+        <v>25900000</v>
       </c>
     </row>
     <row r="11">
@@ -824,10 +824,10 @@
         <v>74</v>
       </c>
       <c r="G11" t="n">
-        <v>45000</v>
+        <v>50000</v>
       </c>
       <c r="H11" t="n">
-        <v>3330000</v>
+        <v>3700000</v>
       </c>
     </row>
     <row r="12">
@@ -860,10 +860,10 @@
         <v>74</v>
       </c>
       <c r="G12" t="n">
-        <v>40000</v>
+        <v>42000</v>
       </c>
       <c r="H12" t="n">
-        <v>2960000</v>
+        <v>3108000</v>
       </c>
     </row>
     <row r="13">
@@ -896,10 +896,10 @@
         <v>74</v>
       </c>
       <c r="G13" t="n">
-        <v>45000</v>
+        <v>50000</v>
       </c>
       <c r="H13" t="n">
-        <v>3330000</v>
+        <v>3700000</v>
       </c>
     </row>
     <row r="14">
@@ -932,10 +932,10 @@
         <v>49.36</v>
       </c>
       <c r="G14" t="n">
-        <v>2500</v>
+        <v>3000</v>
       </c>
       <c r="H14" t="n">
-        <v>123400</v>
+        <v>148080</v>
       </c>
     </row>
     <row r="15">
@@ -968,10 +968,10 @@
         <v>89.56</v>
       </c>
       <c r="G15" t="n">
-        <v>15000</v>
+        <v>16000</v>
       </c>
       <c r="H15" t="n">
-        <v>1343400</v>
+        <v>1432960</v>
       </c>
     </row>
     <row r="16">
@@ -1004,10 +1004,10 @@
         <v>181.58</v>
       </c>
       <c r="G16" t="n">
-        <v>12000</v>
+        <v>13000</v>
       </c>
       <c r="H16" t="n">
-        <v>2178960</v>
+        <v>2360540</v>
       </c>
     </row>
     <row r="17">

</xml_diff>